<commit_message>
Sales unit master product category and product module code
</commit_message>
<xml_diff>
--- a/Documents/CRM_Products.xlsx
+++ b/Documents/CRM_Products.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE8F705A-ACE3-4820-AD03-81896E09B4BD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2721D3E2-3A12-4852-8F08-CE0502941E4C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample Product list" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="163">
   <si>
     <t>Product ID</t>
   </si>
@@ -493,6 +493,21 @@
   </si>
   <si>
     <t>Residential or Business or Both</t>
+  </si>
+  <si>
+    <t>Column2</t>
+  </si>
+  <si>
+    <t>Minimum Period</t>
+  </si>
+  <si>
+    <t>18 Months</t>
+  </si>
+  <si>
+    <t>Default 12 months/18/24</t>
+  </si>
+  <si>
+    <t>Default 24 months/12/18</t>
   </si>
 </sst>
 </file>
@@ -757,7 +772,26 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="32">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -781,10 +815,71 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -801,6 +896,272 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -844,27 +1205,10 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.39997558519241921"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -898,316 +1242,6 @@
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1308,13 +1342,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1332,6 +1359,32 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -1347,40 +1400,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A1:Y25" totalsRowShown="0" headerRowDxfId="13" dataDxfId="29" headerRowBorderDxfId="27" tableBorderDxfId="28" totalsRowBorderDxfId="26">
-  <autoFilter ref="A1:Y25" xr:uid="{00000000-0009-0000-0100-000002000000}">
-    <filterColumn colId="12">
-      <filters>
-        <filter val="mandatory (Yes)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Product ID" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Product/Sevice Name" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Product/service Info" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Provider" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Contact Period" dataDxfId="5"/>
-    <tableColumn id="22" xr3:uid="{F5EC45E6-B669-4FD7-937F-69753236C0E4}" name="Product base price" dataDxfId="4"/>
-    <tableColumn id="23" xr3:uid="{EC054318-48EF-4ADD-B556-25D59F662D4E}" name="Provider base price" dataDxfId="2"/>
-    <tableColumn id="21" xr3:uid="{CF85D6E1-A889-431A-9384-D179BECABBE2}" name="Installment Applicable" dataDxfId="3"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="installmentPay" dataDxfId="21"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="DownPayment" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Product Price" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Order Status" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Bank Info required" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Order Date" dataDxfId="16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table2" displayName="Table2" ref="A1:AA25" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28" totalsRowBorderDxfId="27">
+  <autoFilter ref="A1:AA25" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="27">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Product ID" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Product/Sevice Name" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Product/service Info" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Provider" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Contact Period" dataDxfId="22"/>
+    <tableColumn id="26" xr3:uid="{D568353F-8078-4B88-9648-2FFBDDB104DA}" name="Minimum Period" dataDxfId="1"/>
+    <tableColumn id="27" xr3:uid="{FD81E66B-7CAE-477E-ADF4-4D54E53EE466}" name="Column2" dataDxfId="0"/>
+    <tableColumn id="22" xr3:uid="{F5EC45E6-B669-4FD7-937F-69753236C0E4}" name="Product base price" dataDxfId="21"/>
+    <tableColumn id="23" xr3:uid="{EC054318-48EF-4ADD-B556-25D59F662D4E}" name="Provider base price" dataDxfId="20"/>
+    <tableColumn id="21" xr3:uid="{CF85D6E1-A889-431A-9384-D179BECABBE2}" name="Installment Applicable" dataDxfId="19"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="installmentPay" dataDxfId="18"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="DownPayment" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Product Price" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Order Status" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Bank Info required" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Order Date" dataDxfId="13"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Prodcut?/service Deliverd by" dataDxfId="12"/>
-    <tableColumn id="25" xr3:uid="{C6751AC2-52D4-4E05-ACDB-E57130E4475C}" name="Order confirmation date ( Including third party )" dataDxfId="0"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Product/service Delivery Date ( Delivery date and activation could be different for few products)" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Product/Service Activation Date" dataDxfId="10"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Experiy Date" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Order Cancel date" dataDxfId="8"/>
+    <tableColumn id="25" xr3:uid="{C6751AC2-52D4-4E05-ACDB-E57130E4475C}" name="Order confirmation date ( Including third party )" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Product/service Delivery Date ( Delivery date and activation could be different for few products)" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Product/Service Activation Date" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Experiy Date" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Order Cancel date" dataDxfId="7"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Canceled By" dataDxfId="6"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Comission By 3rd party" dataDxfId="7"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Comission to Agent" dataDxfId="15"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Additional note" dataDxfId="14"/>
-    <tableColumn id="24" xr3:uid="{CD71B688-B414-49E0-9B17-2ED1B79CA8A6}" name="Column1" dataDxfId="1"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Comission By 3rd party" dataDxfId="5"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Comission to Agent" dataDxfId="4"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Additional note" dataDxfId="3"/>
+    <tableColumn id="24" xr3:uid="{CD71B688-B414-49E0-9B17-2ED1B79CA8A6}" name="Column1" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1707,7 +1756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.26953125" style="1" customWidth="1"/>
@@ -1715,26 +1764,26 @@
     <col min="3" max="3" width="21.26953125" style="1" customWidth="1"/>
     <col min="4" max="4" width="10.7265625" style="1" customWidth="1"/>
     <col min="5" max="5" width="17.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="17.90625" style="1" customWidth="1"/>
-    <col min="9" max="10" width="16.1796875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14.81640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.54296875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="12.81640625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="29.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29.54296875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="30.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="32.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="25" max="16384" width="9.1796875" style="1"/>
+    <col min="6" max="10" width="17.90625" style="1" customWidth="1"/>
+    <col min="11" max="12" width="16.1796875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="14.81640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.54296875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="12.81640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="29.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="29.54296875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="30.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="32.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1750,68 +1799,74 @@
       <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H1" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="I1" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="Q1" s="16" t="s">
+      <c r="S1" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="T1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="16" t="s">
+      <c r="U1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="16" t="s">
+      <c r="V1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="U1" s="16" t="s">
+      <c r="W1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="X1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="Z1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="AA1" s="4" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1" ht="39" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" s="2" customFormat="1" ht="39" x14ac:dyDescent="0.35">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1827,43 +1882,41 @@
       <c r="E2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="25">
-        <v>0</v>
-      </c>
-      <c r="G2" s="25">
+      <c r="F2" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="G2" s="7"/>
+      <c r="H2" s="25">
+        <v>0</v>
+      </c>
+      <c r="I2" s="25">
         <v>1</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="L2" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K2" s="7">
-        <v>0</v>
-      </c>
-      <c r="L2" s="7" t="s">
+      <c r="M2" s="7">
+        <v>0</v>
+      </c>
+      <c r="N2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="O2" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N2" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O2" s="7" t="s">
+      <c r="P2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q2" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R2" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R2" s="7"/>
       <c r="S2" s="17" t="s">
         <v>20</v>
       </c>
@@ -1871,19 +1924,25 @@
         <v>20</v>
       </c>
       <c r="U2" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V2" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W2" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V2" s="7" t="s">
+      <c r="X2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W2" s="7" t="s">
+      <c r="Y2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X2" s="9" t="s">
+      <c r="Z2" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:25" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1899,43 +1958,39 @@
       <c r="E3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="25">
-        <v>0</v>
-      </c>
-      <c r="G3" s="25">
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="25">
+        <v>0</v>
+      </c>
+      <c r="I3" s="25">
         <v>15</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="K3" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="L3" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K3" s="7">
-        <v>0</v>
-      </c>
-      <c r="L3" s="7" t="s">
+      <c r="M3" s="7">
+        <v>0</v>
+      </c>
+      <c r="N3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="O3" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O3" s="7" t="s">
+      <c r="P3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P3" s="7"/>
-      <c r="Q3" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R3" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R3" s="7"/>
       <c r="S3" s="17" t="s">
         <v>20</v>
       </c>
@@ -1943,19 +1998,25 @@
         <v>20</v>
       </c>
       <c r="U3" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V3" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W3" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V3" s="7" t="s">
+      <c r="X3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W3" s="7" t="s">
+      <c r="Y3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X3" s="9" t="s">
+      <c r="Z3" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:25" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A4" s="21">
         <v>3</v>
       </c>
@@ -1971,43 +2032,39 @@
       <c r="E4" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="25">
-        <v>0</v>
-      </c>
-      <c r="G4" s="25">
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="25">
+        <v>0</v>
+      </c>
+      <c r="I4" s="25">
         <v>12</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="J4" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="K4" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="L4" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K4" s="7">
-        <v>0</v>
-      </c>
-      <c r="L4" s="7" t="s">
+      <c r="M4" s="7">
+        <v>0</v>
+      </c>
+      <c r="N4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M4" s="7" t="s">
+      <c r="O4" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O4" s="7" t="s">
+      <c r="P4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R4" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R4" s="7"/>
       <c r="S4" s="17" t="s">
         <v>20</v>
       </c>
@@ -2015,19 +2072,25 @@
         <v>20</v>
       </c>
       <c r="U4" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V4" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V4" s="7" t="s">
+      <c r="X4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W4" s="7" t="s">
+      <c r="Y4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X4" s="9" t="s">
+      <c r="Z4" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:25" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A5" s="21">
         <v>4</v>
       </c>
@@ -2043,63 +2106,65 @@
       <c r="E5" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="25">
-        <v>0</v>
-      </c>
-      <c r="G5" s="25">
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="25">
+        <v>0</v>
+      </c>
+      <c r="I5" s="25">
         <v>250</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="J5" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="K5" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="L5" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="M5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="N5" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M5" s="7" t="s">
+      <c r="O5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="N5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O5" s="7" t="s">
+      <c r="P5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R5" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R5" s="7"/>
       <c r="S5" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T5" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="U5" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="T5" s="17" t="s">
+      <c r="V5" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="U5" s="17" t="s">
+      <c r="W5" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="X5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W5" s="7" t="s">
+      <c r="Y5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X5" s="9" t="s">
+      <c r="Z5" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:25" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A6" s="23">
         <v>5</v>
       </c>
@@ -2115,43 +2180,39 @@
       <c r="E6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="25">
-        <v>0</v>
-      </c>
-      <c r="G6" s="25">
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="25">
+        <v>0</v>
+      </c>
+      <c r="I6" s="25">
         <v>12</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="J6" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="K6" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="L6" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K6" s="7">
-        <v>0</v>
-      </c>
-      <c r="L6" s="7" t="s">
+      <c r="M6" s="7">
+        <v>0</v>
+      </c>
+      <c r="N6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="O6" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O6" s="7" t="s">
+      <c r="P6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q6" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R6" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R6" s="7"/>
       <c r="S6" s="17" t="s">
         <v>20</v>
       </c>
@@ -2159,19 +2220,25 @@
         <v>20</v>
       </c>
       <c r="U6" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V6" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W6" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V6" s="7" t="s">
+      <c r="X6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W6" s="7" t="s">
+      <c r="Y6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X6" s="9" t="s">
+      <c r="Z6" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:25" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A7" s="23">
         <v>6</v>
       </c>
@@ -2187,63 +2254,65 @@
       <c r="E7" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="25">
-        <v>0</v>
-      </c>
-      <c r="G7" s="25">
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="25">
+        <v>0</v>
+      </c>
+      <c r="I7" s="25">
         <v>250</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="K7" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J7" s="7">
-        <v>0</v>
-      </c>
-      <c r="K7" s="7" t="s">
+      <c r="L7" s="7">
+        <v>0</v>
+      </c>
+      <c r="M7" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="N7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M7" s="7" t="s">
+      <c r="O7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="N7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O7" s="7" t="s">
+      <c r="P7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q7" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R7" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R7" s="7"/>
       <c r="S7" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T7" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="U7" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="T7" s="17" t="s">
+      <c r="V7" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="U7" s="17" t="s">
+      <c r="W7" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V7" s="7" t="s">
+      <c r="X7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W7" s="7" t="s">
+      <c r="Y7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X7" s="9" t="s">
+      <c r="Z7" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:25" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:27" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -2259,43 +2328,39 @@
       <c r="E8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="25">
-        <v>0</v>
-      </c>
-      <c r="G8" s="25">
-        <v>0</v>
-      </c>
-      <c r="H8" s="7" t="s">
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="25">
+        <v>0</v>
+      </c>
+      <c r="I8" s="25">
+        <v>0</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="K8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="L8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="M8" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L8" s="7" t="s">
+      <c r="N8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M8" s="7" t="s">
+      <c r="O8" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O8" s="7" t="s">
+      <c r="P8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q8" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R8" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R8" s="7"/>
       <c r="S8" s="17" t="s">
         <v>20</v>
       </c>
@@ -2303,22 +2368,28 @@
         <v>20</v>
       </c>
       <c r="U8" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V8" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W8" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V8" s="7" t="s">
+      <c r="X8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W8" s="7" t="s">
+      <c r="Y8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X8" s="9" t="s">
+      <c r="Z8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Y8" s="2" t="s">
+      <c r="AA8" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="9" spans="1:25" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:27" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -2332,45 +2403,41 @@
         <v>41</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="25">
-        <v>0</v>
-      </c>
-      <c r="G9" s="25">
-        <v>0</v>
-      </c>
-      <c r="H9" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="25">
+        <v>0</v>
+      </c>
+      <c r="I9" s="25">
+        <v>0</v>
+      </c>
+      <c r="J9" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="K9" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="L9" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="M9" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L9" s="7" t="s">
+      <c r="N9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="7" t="s">
+      <c r="O9" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O9" s="7" t="s">
+      <c r="P9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R9" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R9" s="7"/>
       <c r="S9" s="17" t="s">
         <v>20</v>
       </c>
@@ -2378,22 +2445,28 @@
         <v>20</v>
       </c>
       <c r="U9" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V9" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W9" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V9" s="7" t="s">
+      <c r="X9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W9" s="7" t="s">
+      <c r="Y9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X9" s="9" t="s">
+      <c r="Z9" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Y9" s="2" t="s">
+      <c r="AA9" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:25" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:27" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -2407,45 +2480,41 @@
         <v>50</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F10" s="25">
-        <v>0</v>
-      </c>
-      <c r="G10" s="25">
-        <v>0</v>
-      </c>
-      <c r="H10" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="25">
+        <v>0</v>
+      </c>
+      <c r="I10" s="25">
+        <v>0</v>
+      </c>
+      <c r="J10" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="K10" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="L10" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="M10" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="L10" s="7" t="s">
+      <c r="N10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M10" s="7" t="s">
+      <c r="O10" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O10" s="7" t="s">
+      <c r="P10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q10" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R10" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R10" s="7"/>
       <c r="S10" s="17" t="s">
         <v>20</v>
       </c>
@@ -2453,22 +2522,28 @@
         <v>20</v>
       </c>
       <c r="U10" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V10" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W10" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V10" s="7" t="s">
+      <c r="X10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W10" s="7" t="s">
+      <c r="Y10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X10" s="9" t="s">
+      <c r="Z10" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Y10" s="2" t="s">
+      <c r="AA10" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="11" spans="1:25" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:27" s="2" customFormat="1" ht="91" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -2482,45 +2557,41 @@
         <v>50</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="25">
-        <v>0</v>
-      </c>
-      <c r="G11" s="25">
-        <v>0</v>
-      </c>
-      <c r="H11" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="25">
+        <v>0</v>
+      </c>
+      <c r="I11" s="25">
+        <v>0</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="K11" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J11" s="7" t="s">
+      <c r="L11" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="K11" s="7" t="s">
+      <c r="M11" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="L11" s="7" t="s">
+      <c r="N11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M11" s="7" t="s">
+      <c r="O11" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N11" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O11" s="7" t="s">
+      <c r="P11" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q11" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R11" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R11" s="7"/>
       <c r="S11" s="17" t="s">
         <v>20</v>
       </c>
@@ -2528,22 +2599,28 @@
         <v>20</v>
       </c>
       <c r="U11" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="V11" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W11" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="V11" s="7" t="s">
+      <c r="X11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="W11" s="7" t="s">
+      <c r="Y11" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X11" s="9" t="s">
+      <c r="Z11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Y11" s="2" t="s">
+      <c r="AA11" s="2" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="12" spans="1:25" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -2559,63 +2636,65 @@
       <c r="E12" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="25">
         <v>7.5</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="I12" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="J12" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="K12" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="L12" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="M12" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="L12" s="7" t="s">
+      <c r="N12" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M12" s="7" t="s">
+      <c r="O12" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O12" s="7" t="s">
+      <c r="P12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q12" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R12" s="17" t="s">
+      <c r="R12" s="7"/>
+      <c r="S12" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T12" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="S12" s="17" t="s">
+      <c r="U12" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="T12" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="U12" s="17" t="s">
+      <c r="V12" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W12" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="V12" s="7" t="s">
+      <c r="X12" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W12" s="7" t="s">
+      <c r="Y12" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X12" s="9" t="s">
+      <c r="Z12" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:25" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
         <v>11</v>
       </c>
@@ -2631,63 +2710,65 @@
       <c r="E13" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="25">
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="25">
         <v>28</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="I13" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="J13" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="K13" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="L13" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="K13" s="7" t="s">
+      <c r="M13" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="L13" s="7" t="s">
+      <c r="N13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M13" s="7" t="s">
+      <c r="O13" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N13" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O13" s="7" t="s">
+      <c r="P13" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q13" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R13" s="17" t="s">
+      <c r="R13" s="7"/>
+      <c r="S13" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T13" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="S13" s="17" t="s">
+      <c r="U13" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="T13" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="U13" s="17" t="s">
+      <c r="V13" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W13" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="V13" s="7" t="s">
+      <c r="X13" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W13" s="7" t="s">
+      <c r="Y13" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X13" s="9" t="s">
+      <c r="Z13" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:25" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
         <v>11</v>
       </c>
@@ -2703,63 +2784,65 @@
       <c r="E14" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="F14" s="25">
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="25">
         <v>18</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="I14" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="J14" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="K14" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="L14" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="M14" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="L14" s="7" t="s">
+      <c r="N14" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="O14" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N14" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O14" s="7" t="s">
+      <c r="P14" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q14" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R14" s="17" t="s">
+      <c r="R14" s="7"/>
+      <c r="S14" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T14" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="S14" s="17" t="s">
+      <c r="U14" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="T14" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="U14" s="17" t="s">
+      <c r="V14" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="W14" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="V14" s="7" t="s">
+      <c r="X14" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W14" s="7" t="s">
+      <c r="Y14" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X14" s="9" t="s">
+      <c r="Z14" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:25" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -2775,63 +2858,65 @@
       <c r="E15" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="25">
         <v>399</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="I15" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="J15" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="K15" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="L15" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="K15" s="7" t="s">
+      <c r="M15" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="L15" s="7" t="s">
+      <c r="N15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M15" s="7" t="s">
+      <c r="O15" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N15" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O15" s="7" t="s">
+      <c r="P15" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q15" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R15" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R15" s="7"/>
       <c r="S15" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T15" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="U15" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="T15" s="17" t="s">
+      <c r="V15" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="U15" s="17" t="s">
+      <c r="W15" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="V15" s="7" t="s">
+      <c r="X15" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W15" s="7" t="s">
+      <c r="Y15" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X15" s="9" t="s">
+      <c r="Z15" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:25" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:27" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -2847,63 +2932,65 @@
       <c r="E16" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="25">
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="25">
         <v>750</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="I16" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="J16" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="K16" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="L16" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="M16" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="L16" s="7" t="s">
+      <c r="N16" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="O16" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N16" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O16" s="7" t="s">
+      <c r="P16" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q16" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R16" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R16" s="7"/>
       <c r="S16" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T16" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="U16" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="T16" s="17" t="s">
+      <c r="V16" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="U16" s="17" t="s">
+      <c r="W16" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="V16" s="7" t="s">
+      <c r="X16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W16" s="7" t="s">
+      <c r="Y16" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X16" s="9" t="s">
+      <c r="Z16" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:24" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -2919,63 +3006,65 @@
       <c r="E17" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="25">
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="25">
         <v>399</v>
       </c>
-      <c r="G17" s="25" t="s">
+      <c r="I17" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="J17" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="K17" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="J17" s="7" t="s">
+      <c r="L17" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="K17" s="7" t="s">
+      <c r="M17" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="L17" s="7" t="s">
+      <c r="N17" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M17" s="7" t="s">
+      <c r="O17" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N17" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O17" s="7" t="s">
+      <c r="P17" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q17" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R17" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R17" s="7"/>
       <c r="S17" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="T17" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="U17" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="V17" s="7" t="s">
+      <c r="V17" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="W17" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="X17" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W17" s="7" t="s">
+      <c r="Y17" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X17" s="9" t="s">
+      <c r="Z17" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:24" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:26" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -2991,63 +3080,65 @@
       <c r="E18" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="25">
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="25">
         <v>250</v>
       </c>
-      <c r="G18" s="25" t="s">
+      <c r="I18" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="J18" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="K18" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="L18" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="M18" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="L18" s="7" t="s">
+      <c r="N18" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="7" t="s">
+      <c r="O18" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N18" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O18" s="7" t="s">
+      <c r="P18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q18" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R18" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R18" s="7"/>
       <c r="S18" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="T18" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="U18" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="V18" s="7" t="s">
+      <c r="V18" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="W18" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="X18" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W18" s="7" t="s">
+      <c r="Y18" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X18" s="9" t="s">
+      <c r="Z18" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:24" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:26" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -3063,63 +3154,65 @@
       <c r="E19" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F19" s="25">
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="25">
         <v>300</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="I19" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="J19" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="K19" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="L19" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="K19" s="7" t="s">
+      <c r="M19" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="L19" s="7" t="s">
+      <c r="N19" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M19" s="7" t="s">
+      <c r="O19" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N19" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O19" s="7" t="s">
+      <c r="P19" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q19" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R19" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R19" s="7"/>
       <c r="S19" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="T19" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="U19" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="V19" s="7" t="s">
+      <c r="V19" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="W19" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="X19" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W19" s="7" t="s">
+      <c r="Y19" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X19" s="9" t="s">
+      <c r="Z19" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:24" s="2" customFormat="1" ht="26" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:26" s="2" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -3135,59 +3228,61 @@
       <c r="E20" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F20" s="25">
-        <v>0</v>
-      </c>
-      <c r="G20" s="25" t="s">
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="25">
+        <v>0</v>
+      </c>
+      <c r="I20" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="J20" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7">
-        <v>0</v>
-      </c>
-      <c r="L20" s="7" t="s">
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7">
+        <v>0</v>
+      </c>
+      <c r="N20" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="M20" s="7" t="s">
+      <c r="O20" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="N20" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O20" s="7" t="s">
+      <c r="P20" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q20" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R20" s="17" t="s">
-        <v>20</v>
-      </c>
+      <c r="R20" s="7"/>
       <c r="S20" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="T20" s="17" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="U20" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="V20" s="7" t="s">
+      <c r="V20" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="W20" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="X20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="W20" s="7" t="s">
+      <c r="Y20" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X20" s="9" t="s">
+      <c r="Z20" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:26" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -3201,65 +3296,67 @@
         <v>93</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="F21" s="26">
-        <v>0</v>
-      </c>
-      <c r="G21" s="26">
-        <v>0</v>
-      </c>
-      <c r="H21" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="26">
+        <v>0</v>
+      </c>
+      <c r="I21" s="26">
+        <v>0</v>
+      </c>
+      <c r="J21" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I21" s="10">
-        <v>0</v>
-      </c>
-      <c r="J21" s="10">
-        <v>0</v>
-      </c>
-      <c r="K21" s="10" t="s">
+      <c r="K21" s="10">
+        <v>0</v>
+      </c>
+      <c r="L21" s="10">
+        <v>0</v>
+      </c>
+      <c r="M21" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="L21" s="10" t="s">
+      <c r="N21" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="M21" s="10" t="s">
+      <c r="O21" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="N21" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O21" s="10" t="s">
+      <c r="P21" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q21" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R21" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="S21" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="T21" s="18" t="s">
+      <c r="R21" s="10"/>
+      <c r="S21" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T21" s="17" t="s">
         <v>20</v>
       </c>
       <c r="U21" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="V21" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="W21" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="V21" s="10" t="s">
+      <c r="X21" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="W21" s="7" t="s">
+      <c r="Y21" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X21" s="11" t="s">
+      <c r="Z21" s="11" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:26" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -3275,63 +3372,65 @@
       <c r="E22" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="F22" s="26">
-        <v>0</v>
-      </c>
-      <c r="G22" s="26">
-        <v>0</v>
-      </c>
-      <c r="H22" s="7" t="s">
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="26">
+        <v>0</v>
+      </c>
+      <c r="I22" s="26">
+        <v>0</v>
+      </c>
+      <c r="J22" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I22" s="10">
-        <v>0</v>
-      </c>
-      <c r="J22" s="10">
-        <v>0</v>
-      </c>
-      <c r="K22" s="10" t="s">
+      <c r="K22" s="10">
+        <v>0</v>
+      </c>
+      <c r="L22" s="10">
+        <v>0</v>
+      </c>
+      <c r="M22" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="L22" s="10" t="s">
+      <c r="N22" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="M22" s="10" t="s">
+      <c r="O22" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="N22" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O22" s="10" t="s">
+      <c r="P22" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q22" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R22" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="S22" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="T22" s="18" t="s">
+      <c r="R22" s="10"/>
+      <c r="S22" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T22" s="17" t="s">
         <v>20</v>
       </c>
       <c r="U22" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="V22" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="W22" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="V22" s="10" t="s">
+      <c r="X22" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="W22" s="7" t="s">
+      <c r="Y22" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X22" s="11" t="s">
+      <c r="Z22" s="11" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -3347,63 +3446,65 @@
       <c r="E23" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="F23" s="26">
-        <v>0</v>
-      </c>
-      <c r="G23" s="26">
-        <v>0</v>
-      </c>
-      <c r="H23" s="7" t="s">
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="26">
+        <v>0</v>
+      </c>
+      <c r="I23" s="26">
+        <v>0</v>
+      </c>
+      <c r="J23" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I23" s="10">
-        <v>0</v>
-      </c>
-      <c r="J23" s="10">
-        <v>0</v>
-      </c>
-      <c r="K23" s="10" t="s">
+      <c r="K23" s="10">
+        <v>0</v>
+      </c>
+      <c r="L23" s="10">
+        <v>0</v>
+      </c>
+      <c r="M23" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="L23" s="10" t="s">
+      <c r="N23" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="M23" s="10" t="s">
+      <c r="O23" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="N23" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O23" s="10" t="s">
+      <c r="P23" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q23" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="P23" s="10"/>
-      <c r="Q23" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R23" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="S23" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="T23" s="18" t="s">
+      <c r="R23" s="10"/>
+      <c r="S23" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T23" s="17" t="s">
         <v>20</v>
       </c>
       <c r="U23" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="V23" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="W23" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="V23" s="10" t="s">
+      <c r="X23" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="W23" s="7" t="s">
+      <c r="Y23" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X23" s="11" t="s">
+      <c r="Z23" s="11" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -3419,63 +3520,65 @@
       <c r="E24" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="F24" s="26">
-        <v>0</v>
-      </c>
-      <c r="G24" s="26">
-        <v>0</v>
-      </c>
-      <c r="H24" s="7" t="s">
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="26">
+        <v>0</v>
+      </c>
+      <c r="I24" s="26">
+        <v>0</v>
+      </c>
+      <c r="J24" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I24" s="10">
-        <v>0</v>
-      </c>
-      <c r="J24" s="10">
-        <v>0</v>
-      </c>
-      <c r="K24" s="10" t="s">
+      <c r="K24" s="10">
+        <v>0</v>
+      </c>
+      <c r="L24" s="10">
+        <v>0</v>
+      </c>
+      <c r="M24" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="L24" s="10" t="s">
+      <c r="N24" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="M24" s="10" t="s">
+      <c r="O24" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="N24" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="O24" s="10" t="s">
+      <c r="P24" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q24" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="R24" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="S24" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="T24" s="18" t="s">
+      <c r="R24" s="10"/>
+      <c r="S24" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T24" s="17" t="s">
         <v>20</v>
       </c>
       <c r="U24" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="V24" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="W24" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="V24" s="10" t="s">
+      <c r="X24" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="W24" s="7" t="s">
+      <c r="Y24" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="X24" s="11" t="s">
+      <c r="Z24" s="11" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:26" ht="29" x14ac:dyDescent="0.35">
       <c r="A25" s="12">
         <v>24</v>
       </c>
@@ -3491,59 +3594,61 @@
       <c r="E25" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="F25" s="26">
-        <v>0</v>
-      </c>
-      <c r="G25" s="27">
-        <v>0</v>
-      </c>
-      <c r="H25" s="7" t="s">
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="26">
+        <v>0</v>
+      </c>
+      <c r="I25" s="27">
+        <v>0</v>
+      </c>
+      <c r="J25" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I25" s="13">
-        <v>0</v>
-      </c>
-      <c r="J25" s="13">
-        <v>0</v>
-      </c>
-      <c r="K25" s="13" t="s">
+      <c r="K25" s="13">
+        <v>0</v>
+      </c>
+      <c r="L25" s="13">
+        <v>0</v>
+      </c>
+      <c r="M25" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="L25" s="13" t="s">
+      <c r="N25" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="M25" s="13" t="s">
+      <c r="O25" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="N25" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="O25" s="13" t="s">
+      <c r="P25" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q25" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="R25" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="S25" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="T25" s="20" t="s">
+      <c r="R25" s="13"/>
+      <c r="S25" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="T25" s="19" t="s">
         <v>20</v>
       </c>
       <c r="U25" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="V25" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="W25" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="V25" s="13" t="s">
+      <c r="X25" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="W25" s="14" t="s">
+      <c r="Y25" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="X25" s="15" t="s">
+      <c r="Z25" s="15" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Agent management module done
</commit_message>
<xml_diff>
--- a/Documents/CRM_Products.xlsx
+++ b/Documents/CRM_Products.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E4272A-887B-476F-A6CE-47CD2F806244}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7A3899-541C-4872-BE0F-CABD01B2E83D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="165">
   <si>
     <t>Product ID</t>
   </si>
@@ -509,6 +509,12 @@
   </si>
   <si>
     <t>Item name</t>
+  </si>
+  <si>
+    <t>World pay</t>
+  </si>
+  <si>
+    <t>Card machine world pay($1 Package)</t>
   </si>
 </sst>
 </file>
@@ -2871,7 +2877,7 @@
         <v>95</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="L15" s="7" t="s">
         <v>84</v>
@@ -3664,11 +3670,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{817B9753-2E78-459D-A301-69C01045B183}">
-  <dimension ref="A2:B2"/>
+  <dimension ref="A2:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -3677,6 +3683,14 @@
       </c>
       <c r="B2" t="s">
         <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>